<commit_message>
feat: add Thai interpretation column to F1 reports
</commit_message>
<xml_diff>
--- a/output/SNOMED/LLM_Evaluation_Report.xlsx
+++ b/output/SNOMED/LLM_Evaluation_Report.xlsx
@@ -666,7 +666,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Troponin measurement (procedure)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -675,14 +675,14 @@
         </is>
       </c>
       <c r="D9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Histopathology test (procedure)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -703,14 +703,14 @@
         </is>
       </c>
       <c r="D10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Calculation of quantitative glomerular filtration rate based on creatinine concentration in serum or plasma (procedure)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -787,14 +787,14 @@
         </is>
       </c>
       <c r="D13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Gene rearrangement analysis (procedure)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -899,14 +899,14 @@
         </is>
       </c>
       <c r="D17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Blastomyces dermatitidis antigen assay (procedure)</t>
+          <t>Measurement of microbial nucleic acid (procedure)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Stool culture for bacteria (procedure)</t>
+          <t>Microbial culture (procedure)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Bacterial culture (procedure)</t>
+          <t>Microbial culture (procedure)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Histopathology test (procedure)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1907,14 +1907,14 @@
         </is>
       </c>
       <c r="D53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Calculation of quantitative glomerular filtration rate based on creatinine concentration in serum or plasma (procedure)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2103,14 +2103,14 @@
         </is>
       </c>
       <c r="D60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Gastric surgical biopsy (procedure)</t>
+          <t>Laboratory test (procedure)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Beta globin gene mutation analysis (procedure)</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3559,14 +3559,14 @@
         </is>
       </c>
       <c r="D112" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E112" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3718,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Scraping of corneal epithelium (procedure)</t>
+          <t>Gram stain microscopy (procedure)</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3998,7 +3998,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Blood compatibility test, crossmatch by incubation technique (procedure)</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -4007,14 +4007,14 @@
         </is>
       </c>
       <c r="D128" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E128" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4110,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Genetic analysis of PKD1 and PKD2 genes (procedure)</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -4119,14 +4119,14 @@
         </is>
       </c>
       <c r="D132" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E132" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Serologic test for syphilis (procedure)</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -4399,14 +4399,14 @@
         </is>
       </c>
       <c r="D142" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E142" t="b">
         <v>0</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>False Positive</t>
         </is>
       </c>
     </row>
@@ -4418,7 +4418,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Laboratory test (procedure)</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -4427,14 +4427,14 @@
         </is>
       </c>
       <c r="D143" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E143" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Examination for suspected tuberculosis (procedure)</t>
+          <t>Microbial culture (procedure)</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -4670,7 +4670,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Antibody measurement (procedure)</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -4679,14 +4679,14 @@
         </is>
       </c>
       <c r="D152" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E152" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -4698,7 +4698,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SMN1 gene deletion analysis (procedure)</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -4707,14 +4707,14 @@
         </is>
       </c>
       <c r="D153" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E153" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -4838,7 +4838,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Blood gas analysis (procedure)</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -4847,14 +4847,14 @@
         </is>
       </c>
       <c r="D158" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E158" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -4950,7 +4950,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Calculation of quantitative glomerular filtration rate based on creatinine concentration in serum or plasma (procedure)</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -4959,14 +4959,14 @@
         </is>
       </c>
       <c r="D162" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E162" t="b">
         <v>0</v>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>False Positive</t>
         </is>
       </c>
     </row>
@@ -5006,7 +5006,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Calculation of quantitative glomerular filtration rate based on creatinine concentration in serum or plasma (procedure)</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -5015,14 +5015,14 @@
         </is>
       </c>
       <c r="D164" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E164" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -5034,7 +5034,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Histopathology test (procedure)</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -5043,14 +5043,14 @@
         </is>
       </c>
       <c r="D165" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E165" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -5062,7 +5062,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Total immunoglobulin measurement (procedure)</t>
+          <t>Immunoglobulin E measurement (procedure)</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -5146,7 +5146,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Virus identification by tissue culture inoculation and observation (procedure)</t>
+          <t>Microbial culture (procedure)</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Heaf test (procedure)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -5323,14 +5323,14 @@
         </is>
       </c>
       <c r="D175" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E175" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>True Positive</t>
+          <t>False Negative</t>
         </is>
       </c>
     </row>
@@ -5538,7 +5538,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Human immunodeficiency virus type 2 confirmatory assay (procedure)</t>
+          <t>Human immunodeficiency virus screening (procedure)</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Calculation of quantitative glomerular filtration rate based on creatinine concentration in serum or plasma (procedure)</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -6023,14 +6023,14 @@
         </is>
       </c>
       <c r="D200" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E200" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>False Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6092,6 +6092,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Interpretation (คำแปลผล)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6100,11 +6105,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>AI mapped correctly and Expert agreed</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AI จับคู่รหัสได้ถูกต้องและปลอดภัยตามหลักการแพทย์</t>
         </is>
       </c>
     </row>
@@ -6115,11 +6125,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>AI mapped it, but Expert says it is wrong (Hallucination)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AI จับคู่มาให้ แต่ผิดสเปค (อาการ AI หลอน)</t>
         </is>
       </c>
     </row>
@@ -6137,6 +6152,11 @@
           <t>AI left it unmapped (-), and Expert agreed it should be unmapped</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>หมอสั่งกำกวม ระบบจึงปัดเป็นค่าว่าง (-) ซึ่งเป็นการตัดสินใจที่ถูกต้องและปลอดภัยแล้ว</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6145,11 +6165,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>AI left it unmapped (-), but Expert says it could have been mapped</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ระบบเซฟตี้ตัวเองโดยการปัดเป็นค่าว่าง (-) ทั้งที่จริงๆ แล้วถ้าพยายามเดาก็อาจจะหาคู่เจอ</t>
         </is>
       </c>
     </row>
@@ -6161,12 +6186,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.9763</t>
+          <t>0.9677</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>Accuracy of positive predictions (TP / (TP + FP))</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ความแม่นยำ: ถ้า AI จับคู่รหัสมาให้ โอกาสที่จะถูกต้องและนำไปใช้ได้จริงมีสูงถึง 96.77%</t>
         </is>
       </c>
     </row>
@@ -6178,12 +6208,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.8967</t>
+          <t>0.9890</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>Ability to find all valid mappings (TP / (TP + FN))</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ความครอบคลุม: จากรหัสทั้งหมดที่ควรจะจับคู่ได้ ระบบสามารถตามเก็บกวาดมาได้ 98.90%</t>
         </is>
       </c>
     </row>
@@ -6195,12 +6230,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.9348</t>
+          <t>0.9783</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>Harmonic mean of Precision and Recall</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>คะแนนภาพรวม: ระบบมีความสมดุลทั้งความแม่นยำและความครอบคลุมอยู่ในเกณฑ์ดีเยี่ยม (97.83%)</t>
         </is>
       </c>
     </row>

</xml_diff>